<commit_message>
Add SERP data for 5 remaining categories; rebuild archive
Wire SERP 100-104 (colposcopes, surgical lasers, ENT chairs, endoscopy stacks,
UPS for ultrasound) into the 5 previously SERP-less category files and rebuild
medford_categories_all.zip.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Rw9dvcAKokoAsKsBSt35U
</commit_message>
<xml_diff>
--- a/medford_endoskopicheskie_stoyki.xlsx
+++ b/medford_endoskopicheskie_stoyki.xlsx
@@ -941,7 +941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1188,6 +1188,82 @@
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>FAQ_06</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Что такое эндоскопическая стойка?</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Зависит от модели и клинической задачи. Подберём вариант под ваши требования и ответим на вопрос при консультации — напишите или позвоните: +7 (499) 495-48-21.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>endoskopicheskie_stoyki</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>FAQ_07</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>170</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Сколько стоит эндоскопическая стойка?</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Зависит от модели и клинической задачи. Подберём вариант под ваши требования и ответим на вопрос при консультации — напишите или позвоните: +7 (499) 495-48-21.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>endoskopicheskie_stoyki</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>

</xml_diff>